<commit_message>
feat(rq3): FP/FN delta sheet with parsed_label (TEMP) column for spot-check
Emits only the genuinely-new rows vs the reviewed v1 frame so human re-review is
minimal (22 rows). Adds parsed_label (TEMP) at col G (vulnerable/safe) matching the
v1 sheet so the reviewer checks the parsed label against the response text. Identity
compared frame-vs-frame on untruncated (source_code, response_text) to avoid Excel
cell-truncation false mismatches (had inflated the count to 26/39).
</commit_message>
<xml_diff>
--- a/results/rq3_baseline/fpfn_rater_sheet_v2_delta.xlsx
+++ b/results/rq3_baseline/fpfn_rater_sheet_v2_delta.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,21 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDDDDD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -416,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -425,11 +436,12 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,35 +477,40 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>parsed_label (TEMP)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>completeness_score</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>clarity_score</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>actionability_score</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>informativeness_score</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>rater_notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>static struct dir *squashfs_opendir(unsigned int block_start, unsigned int offset,
 	struct inode **i)
@@ -593,22 +610,22 @@
 }</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>['CWE-200']</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>squashfs_opendir in unsquash-2.c in Squashfs-Tools 4.5 allows Directory Traversal, a different vulnerability than CVE-2021-40153. A squashfs filesystem that has been crafted to include a symbolic link and then contents under the same filename in a filesystem can cause unsquashfs to first create the symbolic link pointing outside the expected directory, and then the subsequent write operation will cause the unsquashfs process to write through the symbolic link elsewhere in the filesystem.</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step by step to determine whether there is a vulnerability.
 ---
@@ -840,17 +857,22 @@
 The code is safe from memory corruption and exploitation, despite a minor logic error in the loop condition.</t>
         </is>
       </c>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>static s32 svc_parse_slice(GF_BitStream *bs, AVCState *avc, AVCSliceInfo *si)
 {
@@ -898,14 +920,14 @@
 }</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -922,17 +944,22 @@
 Answer: (1) YES</t>
         </is>
       </c>
-      <c r="G3" s="1" t="n"/>
-      <c r="H3" s="1" t="n"/>
-      <c r="I3" s="1" t="n"/>
-      <c r="J3" s="1" t="n"/>
-      <c r="K3" s="1" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>change_indent(
     int		type,
@@ -1122,14 +1149,14 @@
 }</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n"/>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Code Overview**
@@ -1154,17 +1181,22 @@
 **Note:** This analysis is based on the provided code snippet and assumes the surrounding code and environment do not mitigate the identified concerns. A full audit of the entire codebase would be necessary for a comprehensive vulnerability assessment.</t>
         </is>
       </c>
-      <c r="G4" s="1" t="n"/>
-      <c r="H4" s="1" t="n"/>
-      <c r="I4" s="1" t="n"/>
-      <c r="J4" s="1" t="n"/>
-      <c r="K4" s="1" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>72</v>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>suggest_trie_walk(
     suginfo_T	*su,
@@ -2245,14 +2277,14 @@
 		mch_memmove(p + fl + tl, p</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n"/>
-      <c r="E5" s="1" t="n"/>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>**Step-by-Step Analysis**
 Given the provided code snippet, which appears to be a part of a spell checking or suggestion system (likely from Vim, given the style and some function names), we will analyze it for potential vulnerabilities.
@@ -2282,17 +2314,22 @@
 - Ensure all string operations use length-limited functions (e.g., `strncpy` instead of `strcpy`).</t>
         </is>
       </c>
-      <c r="G5" s="1" t="n"/>
-      <c r="H5" s="1" t="n"/>
-      <c r="I5" s="1" t="n"/>
-      <c r="J5" s="1" t="n"/>
-      <c r="K5" s="1" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>96</v>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>static void build_dirs(char *src, char *dst, size_t src_prefix_len, size_t dst_prefix_len) {
 	char *p = src + src_prefix_len + 1;
@@ -2331,14 +2368,14 @@
 }</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Functionality Overview**
@@ -2382,17 +2419,22 @@
 **Result: (1) YES: Vulnerability detected.**</t>
         </is>
       </c>
-      <c r="G6" s="1" t="n"/>
-      <c r="H6" s="1" t="n"/>
-      <c r="I6" s="1" t="n"/>
-      <c r="J6" s="1" t="n"/>
-      <c r="K6" s="1" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>static s32 svc_parse_slice(GF_BitStream *bs, AVCState *avc, AVCSliceInfo *si)
 {
@@ -2440,14 +2482,14 @@
 }</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n"/>
-      <c r="E7" s="1" t="n"/>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a **static program analysis** and **security vulnerability detection** perspective.
 ---
@@ -2574,17 +2616,22 @@
 **(1) YES: Vulnerability detected.**</t>
         </is>
       </c>
-      <c r="G7" s="1" t="n"/>
-      <c r="H7" s="1" t="n"/>
-      <c r="I7" s="1" t="n"/>
-      <c r="J7" s="1" t="n"/>
-      <c r="K7" s="1" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>119</v>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>gpg_ctx_add_recipient (struct _GpgCtx *gpg,
                        const gchar *keyid)
@@ -2597,22 +2644,22 @@
 }</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>['CWE-200']</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>The gpg_ctx_add_recipient function in camel/camel-gpg-context.c in GNOME Evolution 3.8.4 and earlier and Evolution Data Server 3.9.5 and earlier does not properly select the GPG key to use for email encryption, which might cause the email to be encrypted with the wrong key and allow remote attackers to obtain sensitive information.</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>After analyzing the provided code, I conclude that it **is vulnerable**. Here's the step-by-step reasoning:
 ### 1. **Input Validation Issue**
@@ -2638,17 +2685,22 @@
 **Answer: (1) YES**</t>
         </is>
       </c>
-      <c r="G8" s="1" t="n"/>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
-      <c r="J8" s="1" t="n"/>
-      <c r="K8" s="1" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>131</v>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>static size_t copy_page_to_iter_pipe(struct page *page, size_t offset, size_t bytes,
 			 struct iov_iter *i)
@@ -2693,22 +2745,22 @@
 }</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>['CWE-284']</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>A flaw was found in the way the "flags" member of the new pipe buffer structure was lacking proper initialization in copy_page_to_iter_pipe and push_pipe functions in the Linux kernel and could thus contain stale values. An unprivileged local user could use this flaw to write to pages in the page cache backed by read only files and as such escalate their privileges on the system.</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
@@ -2738,17 +2790,22 @@
 **(2) NO: No vulnerability.** (Within the scope of the provided code snippet and typical static analysis for common vulnerabilities like buffer overflows, use-after-free, etc.)</t>
         </is>
       </c>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="1" t="n"/>
-      <c r="J9" s="1" t="n"/>
-      <c r="K9" s="1" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>161</v>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>static void build_dirs(char *src, char *dst, size_t src_prefix_len, size_t dst_prefix_len) {
 	char *p = src + src_prefix_len + 1;
@@ -2787,14 +2844,14 @@
 }</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n"/>
-      <c r="E10" s="1" t="n"/>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -2809,17 +2866,22 @@
 (1) YES: Vulnerability detected.</t>
         </is>
       </c>
-      <c r="G10" s="1" t="n"/>
-      <c r="H10" s="1" t="n"/>
-      <c r="I10" s="1" t="n"/>
-      <c r="J10" s="1" t="n"/>
-      <c r="K10" s="1" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>189</v>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>static sctp_disposition_t sctp_sf_violation_paramlen(
 				     const struct sctp_endpoint *ep,
@@ -2833,22 +2895,22 @@
 }</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>['CWE-20']</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>The Stream Control Transmission Protocol (sctp) implementation in the Linux kernel before 2.6.27 does not properly handle a protocol violation in which a parameter has an invalid length, which allows attackers to cause a denial of service (panic) via unspecified vectors, related to sctp_sf_violation_paramlen, sctp_sf_abort_violation, sctp_make_abort_violation, and incorrect data types in function calls.</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
@@ -2862,17 +2924,22 @@
 Answer: (2) NO: No vulnerability.</t>
         </is>
       </c>
-      <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="1" t="n"/>
-      <c r="J11" s="1" t="n"/>
-      <c r="K11" s="1" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>197</v>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>static bool tipc_crypto_key_rcv(struct tipc_crypto *rx, struct tipc_msg *hdr)
 {
@@ -2926,14 +2993,14 @@
 }</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
@@ -2957,17 +3024,22 @@
 Answer: (2) NO: No vulnerability.</t>
         </is>
       </c>
-      <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="1" t="n"/>
-      <c r="J12" s="1" t="n"/>
-      <c r="K12" s="1" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>static struct dir *squashfs_opendir(unsigned int block_start, unsigned int offset,
 	struct inode **i)
@@ -3067,22 +3139,22 @@
 }</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>['CWE-200']</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>squashfs_opendir in unsquash-2.c in Squashfs-Tools 4.5 allows Directory Traversal, a different vulnerability than CVE-2021-40153. A squashfs filesystem that has been crafted to include a symbolic link and then contents under the same filename in a filesystem can cause unsquashfs to first create the symbolic link pointing outside the expected directory, and then the subsequent write operation will cause the unsquashfs process to write through the symbolic link elsewhere in the filesystem.</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>After a thorough analysis of the provided code, I have identified no vulnerabilities that would lead to security issues such as buffer overflows, integer overflows causing arbitrary code execution, or other exploitable conditions. Here's the step-by-step reasoning:
 ### Key Checks Performed:
@@ -3116,17 +3188,22 @@
 **Answer: (2) NO**</t>
         </is>
       </c>
-      <c r="G13" s="1" t="n"/>
-      <c r="H13" s="1" t="n"/>
-      <c r="I13" s="1" t="n"/>
-      <c r="J13" s="1" t="n"/>
-      <c r="K13" s="1" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>237</v>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>gpg_ctx_add_recipient (struct _GpgCtx *gpg,
                        const gchar *keyid)
@@ -3139,22 +3216,22 @@
 }</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>['CWE-200']</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>The gpg_ctx_add_recipient function in camel/camel-gpg-context.c in GNOME Evolution 3.8.4 and earlier and Evolution Data Server 3.9.5 and earlier does not properly select the GPG key to use for email encryption, which might cause the email to be encrypted with the wrong key and allow remote attackers to obtain sensitive information.</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step by step to determine whether there is a vulnerability.
 ---
@@ -3228,17 +3305,22 @@
 **(1) YES: Vulnerability detected.**</t>
         </is>
       </c>
-      <c r="G14" s="1" t="n"/>
-      <c r="H14" s="1" t="n"/>
-      <c r="I14" s="1" t="n"/>
-      <c r="J14" s="1" t="n"/>
-      <c r="K14" s="1" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>314</v>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>void add_interrupt_randomness(int irq, int irq_flags)
 {
@@ -3297,22 +3379,22 @@
 }</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>['CWE-200']</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>The Linux kernel through 5.7.11 allows remote attackers to make observations that help to obtain sensitive information about the internal state of the network RNG, aka CID-f227e3ec3b5c. This is related to drivers/char/random.c and kernel/time/timer.c.</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>After a thorough analysis of the provided code, which is part of the Linux kernel's entropy collection mechanism for interrupt handling, I find **no security vulnerability**. Here's the step-by-step reasoning:
 ### Key Observations:
@@ -3347,17 +3429,22 @@
 **Result: (2) NO**</t>
         </is>
       </c>
-      <c r="G15" s="1" t="n"/>
-      <c r="H15" s="1" t="n"/>
-      <c r="I15" s="1" t="n"/>
-      <c r="J15" s="1" t="n"/>
-      <c r="K15" s="1" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>323</v>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>static sctp_disposition_t sctp_sf_violation_paramlen(
 				     const struct sctp_endpoint *ep,
@@ -3371,22 +3458,22 @@
 }</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>['CWE-20']</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>The Stream Control Transmission Protocol (sctp) implementation in the Linux kernel before 2.6.27 does not properly handle a protocol violation in which a parameter has an invalid length, which allows attackers to cause a denial of service (panic) via unspecified vectors, related to sctp_sf_violation_paramlen, sctp_sf_abort_violation, sctp_make_abort_violation, and incorrect data types in function calls.</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if there is a vulnerability present.
 ### Code Snippet:
@@ -3424,107 +3511,22 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
-      <c r="G16" s="1" t="n"/>
-      <c r="H16" s="1" t="n"/>
-      <c r="I16" s="1" t="n"/>
-      <c r="J16" s="1" t="n"/>
-      <c r="K16" s="1" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>327</v>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Result ZipFile::uncompressEntry (int index, const File&amp; targetDirectory, bool shouldOverwriteFiles)
-{
-    auto* zei = entries.getUnchecked (index);
-   #if JUCE_WINDOWS
-    auto entryPath = zei-&gt;entry.filename;
-   #else
-    auto entryPath = zei-&gt;entry.filename.replaceCharacter ('\\', '/');
-   #endif
-    if (entryPath.isEmpty())
-        return Result::ok();
-    auto targetFile = targetDirectory.getChildFile (entryPath);
-    if (entryPath.endsWithChar ('/') || entryPath.endsWithChar ('\\'))
-        return targetFile.createDirectory(); // (entry is a directory, not a file)
-    std::unique_ptr&lt;InputStream&gt; in (createStreamForEntry (index));
-    if (in == nullptr)
-        return Result::fail ("Failed to open the zip file for reading");
-    if (targetFile.exists())
-    {
-        if (! shouldOverwriteFiles)
-            return Result::ok();
-        if (! targetFile.deleteFile())
-            return Result::fail ("Failed to write to target file: " + targetFile.getFullPathName());
-    }
-    if (! targetFile.getParentDirectory().createDirectory())
-        return Result::fail ("Failed to create target folder: " + targetFile.getParentDirectory().getFullPathName());
-    if (zei-&gt;entry.isSymbolicLink)
-    {
-        String originalFilePath (in-&gt;readEntireStreamAsString()
-                                    .replaceCharacter (L'/', File::getSeparatorChar()));
-        if (! File::createSymbolicLink (targetFile, originalFilePath, true))
-            return Result::fail ("Failed to create symbolic link: " + originalFilePath);
-    }
-    else
-    {
-        FileOutputStream out (targetFile);
-        if (out.failedToOpen())
-            return Result::fail ("Failed to write to target file: " + targetFile.getFullPathName());
-        out &lt;&lt; *in;
-    }
-    targetFile.setCreationTime (zei-&gt;entry.fileTime);
-    targetFile.setLastModificationTime (zei-&gt;entry.fileTime);
-    targetFile.setLastAccessTime (zei-&gt;entry.fileTime);
-    return Result::ok();
-}-</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>['CWE-59']</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>This affects the package juce-framework/JUCE before 6.1.5. This vulnerability is triggered when a malicious archive is crafted with an entry containing a symbolic link. When extracted, the symbolic link is followed outside of the target dir allowing writing arbitrary files on the target host. In some cases, this can allow an attacker to execute arbitrary code. The vulnerable code is in the ZipFile::uncompressEntry function in juce_ZipFile.cpp and is executed when the archive is extracted upon calling uncompressTo() on a ZipFile object.</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>YES: Vulnerability detected.
-**Step-by-Step Explanation:**
-1. **Path Traversal Vulnerability:**
-   - The function constructs `targetFile` using `targetDirectory.getChildFile(entryPath)`, where `entryPath` is derived directly from the zip entry's filename.
-   - If the `entryPath` contains directory traversal sequences (e.g., `../../malicious`), `targetFile` will resolve to a path outside the intended `targetDirectory`.
-   - The code does not validate or sanitize `entryPath` to ensure it stays within the target directory, allowing an attacker to write files to arbitrary locations on the system.
-2. **Potential Null Pointer Dereference:**
-   - The use of `entries.getUnchecked(index)` assumes `index` is valid. If `index` is out of bounds (e.g., due to a malformed zip file), `zei` could be a null pointer, leading to a crash when accessing `zei-&gt;entry.filename`.
-3. **Symbolic Link Risks:**
-   - For symbolic links, the target path is read directly from the zip entry's stream without validation. This could allow creation of symlinks to arbitrary locations, potentially leading to privilege escalation or data exposure.
-**Conclusion:** The primary vulnerability is the lack of path traversal checks, enabling attackers to overwrite arbitrary files. This makes the code vulnerable. 
-Answer: YES</t>
-        </is>
-      </c>
-      <c r="G17" s="1" t="n"/>
-      <c r="H17" s="1" t="n"/>
-      <c r="I17" s="1" t="n"/>
-      <c r="J17" s="1" t="n"/>
-      <c r="K17" s="1" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>352</v>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>fiber_switch(mrb_state *mrb, mrb_value self, mrb_int len, const mrb_value *a, mrb_bool resume, mrb_bool vmexec)
 {
@@ -3588,22 +3590,22 @@
 }</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>['CWE-703']</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>NULL Pointer Dereference in GitHub repository mruby/mruby prior to 3.2.</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>### Analysis of the Provided Code
 The function `fiber_switch` is part of a fiber implementation in a language like MRuby, responsible for switching between lightweight threads (fibers). It handles context switching, argument passing, and error checking based on the current state of the fiber.
@@ -3644,246 +3646,22 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
-      <c r="G18" s="1" t="n"/>
-      <c r="H18" s="1" t="n"/>
-      <c r="I18" s="1" t="n"/>
-      <c r="J18" s="1" t="n"/>
-      <c r="K18" s="1" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>361</v>
-      </c>
-      <c r="B19" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Result ZipFile::uncompressEntry (int index, const File&amp; targetDirectory, bool shouldOverwriteFiles)
-{
-    auto* zei = entries.getUnchecked (index);
-   #if JUCE_WINDOWS
-    auto entryPath = zei-&gt;entry.filename;
-   #else
-    auto entryPath = zei-&gt;entry.filename.replaceCharacter ('\\', '/');
-   #endif
-    if (entryPath.isEmpty())
-        return Result::ok();
-    auto targetFile = targetDirectory.getChildFile (entryPath);
-    if (entryPath.endsWithChar ('/') || entryPath.endsWithChar ('\\'))
-        return targetFile.createDirectory(); // (entry is a directory, not a file)
-    std::unique_ptr&lt;InputStream&gt; in (createStreamForEntry (index));
-    if (in == nullptr)
-        return Result::fail ("Failed to open the zip file for reading");
-    if (targetFile.exists())
-    {
-        if (! shouldOverwriteFiles)
-            return Result::ok();
-        if (! targetFile.deleteFile())
-            return Result::fail ("Failed to write to target file: " + targetFile.getFullPathName());
-    }
-    if (! targetFile.getParentDirectory().createDirectory())
-        return Result::fail ("Failed to create target folder: " + targetFile.getParentDirectory().getFullPathName());
-    if (zei-&gt;entry.isSymbolicLink)
-    {
-        String originalFilePath (in-&gt;readEntireStreamAsString()
-                                    .replaceCharacter (L'/', File::getSeparatorChar()));
-        if (! File::createSymbolicLink (targetFile, originalFilePath, true))
-            return Result::fail ("Failed to create symbolic link: " + originalFilePath);
-    }
-    else
-    {
-        FileOutputStream out (targetFile);
-        if (out.failedToOpen())
-            return Result::fail ("Failed to write to target file: " + targetFile.getFullPathName());
-        out &lt;&lt; *in;
-    }
-    targetFile.setCreationTime (zei-&gt;entry.fileTime);
-    targetFile.setLastModificationTime (zei-&gt;entry.fileTime);
-    targetFile.setLastAccessTime (zei-&gt;entry.fileTime);
-    return Result::ok();
-}-</t>
-        </is>
-      </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>['CWE-59']</t>
-        </is>
-      </c>
-      <c r="E19" s="1" t="inlineStr">
-        <is>
-          <t>This affects the package juce-framework/JUCE before 6.1.5. This vulnerability is triggered when a malicious archive is crafted with an entry containing a symbolic link. When extracted, the symbolic link is followed outside of the target dir allowing writing arbitrary files on the target host. In some cases, this can allow an attacker to execute arbitrary code. The vulnerable code is in the ZipFile::uncompressEntry function in juce_ZipFile.cpp and is executed when the archive is extracted upon calling uncompressTo() on a ZipFile object.</t>
-        </is>
-      </c>
-      <c r="F19" s="1" t="inlineStr">
-        <is>
-          <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
-**Code Overview**
-----------------
-The `ZipFile::uncompressEntry` function extracts a specific entry from a ZIP file to a target directory. It handles files, directories, and symbolic links.
-**Step-by-Step Analysis**
--------------------------
-1. **Input Validation**
-	* `index`: Accessed via `entries.getUnchecked(index)`. **Potential Issue**: No bounds checking is shown here. If `index` is out of range, this could lead to undefined behavior.
-	* `targetDirectory`: Assumed valid, but its validity (e.g., being a directory, having write permissions) is checked later.
-	* `shouldOverwriteFiles`: Boolean, no validation issues expected.
-2. **Path Handling**
-	* `entryPath`: Derived from `zei-&gt;entry.filename`. **Potential Issue**: No sanitization is applied to the filename. This could lead to **Path Traversal** vulnerabilities if the filename contains relative paths (e.g., `../../`). However, the use of `targetDirectory.getChildFile(entryPath)` might mitigate this by resolving the path relative to `targetDirectory`.
-3. **Directory Creation**
-	* If `entryPath` ends with a directory separator, it attempts to create a directory. **No immediate issues spotted**.
-4. **File Overwrite Handling**
-	* Checks if `targetFile` exists and handles overwrite logic. **No issues spotted**.
-5. **Parent Directory Creation**
-	* Attempts to create the parent directory if it doesn't exist. **No immediate issues spotted**.
-6. **Symbolic Link Handling**
-	* Reads the link target from the stream and creates a symbolic link. **Potential Issue**: The link target (`originalFilePath`) is read from the ZIP stream and used directly. If an attacker controls the ZIP file, they could create a malicious symbolic link (e.g., pointing to a sensitive system file). However, the `File::createSymbolicLink` with the third parameter set to `true` might indicate a security measure (possibly forcing the link to be within the target directory or resolving it safely).
-7. **File Writing**
-	* Writes the file content from `in` to `out`. **No immediate issues spotted**.
-8. **Time Attribute Setting**
-	* Sets file times from the ZIP entry. **No security issues expected**.
-**Vulnerability Assessment**
----------------------------
-Based on the analysis:
-* **Potential Vulnerability 1**: Lack of bounds checking for `index` in `entries.getUnchecked(index)`.
-* **Potential Vulnerability 2**: Possible Path Traversal through `entryPath` if not properly sanitized, though partially mitigated.
-* **Potential Vulnerability 3**: Symbolic link target resolution might be exploited if `File::createSymbolicLink` with `true` does not adequately sanitize or restrict the link target.
-**Result**
-----------
-Given the potential vulnerabilities identified, especially considering the lack of input sanitization and validation which could lead to security issues:
-**(1) YES: Vulnerability detected.**
-**Recommendations for Improvement**
-1. **Bounds Checking**: Implement bounds checking for `index` before accessing `entries`.
-2. **Path Sanitization**: Sanitize `entryPath` to prevent Path Traversal attacks.
-3. **Symbolic Link Handling**: Ensure `File::createSymbolicLink` with `true` provides sufficient security, or add additional checks for the link target.</t>
-        </is>
-      </c>
-      <c r="G19" s="1" t="n"/>
-      <c r="H19" s="1" t="n"/>
-      <c r="I19" s="1" t="n"/>
-      <c r="J19" s="1" t="n"/>
-      <c r="K19" s="1" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>366</v>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    QueueHandle_t xQueueGenericCreate( const UBaseType_t uxQueueLength,
-                                       const UBaseType_t uxItemSize,
-                                       const uint8_t ucQueueType )
-    {
-        Queue_t * pxNewQueue;
-        size_t xQueueSizeInBytes;
-        uint8_t * pucQueueStorage;
-        configASSERT( uxQueueLength &gt; ( UBaseType_t ) 0 );
-        /* Allocate enough space to hold the maximum number of items that
-         * can be in the queue at any time.  It is valid for uxItemSize to be
-         * zero in the case the queue is used as a semaphore. */
-        xQueueSizeInBytes = ( size_t ) ( uxQueueLength * uxItemSize ); /*lint !e961 MISRA exception as the casts are only redundant for some ports. */
-        /* Check for multiplication overflow. */
-        configASSERT( ( uxItemSize == 0 ) || ( uxQueueLength == ( xQueueSizeInBytes / uxItemSize ) ) );
-        /* Check for addition overflow. */
-        configASSERT( ( sizeof( Queue_t ) + xQueueSizeInBytes ) &gt;  xQueueSizeInBytes );
-        /* Allocate the queue and storage area.  Justification for MISRA
-         * deviation as follows:  pvPortMalloc() always ensures returned memory
-         * blocks are aligned per the requirements of the MCU stack.  In this case
-         * pvPortMalloc() must return a pointer that is guaranteed to meet the
-         * alignment requirements of the Queue_t structure - which in this case
-         * is an int8_t *.  Therefore, whenever the stack alignment requirements
-         * are greater than or equal to the pointer to char requirements the cast
-         * is safe.  In other cases alignment requirements are not strict (one or
-         * two bytes). */
-        pxNewQueue = ( Queue_t * ) pvPortMalloc( sizeof( Queue_t ) + xQueueSizeInBytes ); /*lint !e9087 !e9079 see comment above. */
-        if( pxNewQueue != NULL )
-        {
-            /* Jump past the queue structure to find the location of the queue
-             * storage area. */
-            pucQueueStorage = ( uint8_t * ) pxNewQueue;
-            pucQueueStorage += sizeof( Queue_t ); /*lint !e9016 Pointer arithmetic allowed on char types, especially when it assists conveying intent. */
-            #if ( configSUPPORT_STATIC_ALLOCATION == 1 )
-                {
-                    /* Queues can be created either statically or dynamically, so
-                     * note this task was created dynamically in case it is later
-                     * deleted. */
-                    pxNewQueue-&gt;ucStaticallyAllocated = pdFALSE;
-                }
-            #endif /* configSUPPORT_STATIC_ALLOCATION */
-            prvInitialiseNewQueue( uxQueueLength, uxItemSize, pucQueueStorage, ucQueueType, pxNewQueue );
-        }
-        else
-        {
-            traceQUEUE_CREATE_FAILED( ucQueueType );
-            mtCOVERAGE_TEST_MARKER();
-        }
-        return pxNewQueue;
-    }-</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="n"/>
-      <c r="E20" s="1" t="n"/>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
-**Code Overview**
-----------------
-The function `xQueueGenericCreate` is responsible for creating a queue in a real-time operating system (RTOS) context. It allocates memory for the queue structure and its associated storage area, checks for various types of overflows, and initializes the queue.
-**Step-by-Step Analysis**
--------------------------
-1. **Input Validation**
-	* `uxQueueLength` is validated to be greater than 0 using `configASSERT`.
-	* **No explicit validation for `uxItemSize` or `ucQueueType`**, but:
-		+ `uxItemSize` is used in a way that if it's 0, it's handled as a special case (queue used as a semaphore).
-		+ `ucQueueType` is not validated but is likely constrained by the RTOS's design (e.g., enum values).
-	* **Vulnerability Potential: Low** (assuming `ucQueueType` is constrained by the RTOS)
-2. **Integer Overflows**
-	* **Multiplication Overflow Check**: `configASSERT` checks if `uxQueueLength * uxItemSize` overflows.
-	* **Addition Overflow Check**: `configASSERT` checks if `sizeof(Queue_t) + xQueueSizeInBytes` overflows.
-	* **Vulnerability Potential: NO** (checks are in place)
-3. **Memory Allocation**
-	* Memory is allocated using `pvPortMalloc`, which is assumed to be a safe, RTOS-provided memory allocation function.
-	* **No explicit check for `pvPortMalloc` failure** is shown in the snippet, but:
-		+ The function does check if `pxNewQueue` is `NULL` after allocation.
-	* **Vulnerability Potential: NO** (failure is checked)
-4. **Pointer Arithmetic and Casting**
-	* Pointer arithmetic is used to find the queue storage area. The code includes a **justification for MISRA deviation**, indicating awareness of potential issues.
-	* **Vulnerability Potential: NO** (with the assumption that the RTOS ensures proper alignment)
-5. **Initialization and Error Handling**
-	* The queue is initialized using `prvInitialiseNewQueue` if allocation is successful.
-	* Error handling for allocation failure is present (`traceQUEUE_CREATE_FAILED` and `mtCOVERAGE_TEST_MARKER`).
-	* **Vulnerability Potential: NO**
-**Conclusion**
---------------
-Based on the step-by-step analysis, the code appears to handle potential vulnerabilities adequately:
-* Input validation is partially covered, with assumptions about the RTOS constraining `ucQueueType`.
-* Integer overflows are explicitly checked.
-* Memory allocation failure is handled.
-* Pointer arithmetic and casting are justified with assumptions about the RTOS.
-* Initialization and error handling are in place.
-**Result: (2) NO: No vulnerability.**
-**Note:** This analysis is based on the provided code snippet and assumes the surrounding RTOS environment ensures certain constraints (e.g., on `ucQueueType`, memory alignment). Always consider the broader system context when assessing security.</t>
-        </is>
-      </c>
-      <c r="G20" s="1" t="n"/>
-      <c r="H20" s="1" t="n"/>
-      <c r="I20" s="1" t="n"/>
-      <c r="J20" s="1" t="n"/>
-      <c r="K20" s="1" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>373</v>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>void add_interrupt_randomness(int irq, int irq_flags)
 {
@@ -3942,22 +3720,22 @@
 }</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>['CWE-200']</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>The Linux kernel through 5.7.11 allows remote attackers to make observations that help to obtain sensitive information about the internal state of the network RNG, aka CID-f227e3ec3b5c. This is related to drivers/char/random.c and kernel/time/timer.c.</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step by step to determine whether there is a vulnerability.
 ---
@@ -4088,17 +3866,22 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
-      <c r="G21" s="1" t="n"/>
-      <c r="H21" s="1" t="n"/>
-      <c r="I21" s="1" t="n"/>
-      <c r="J21" s="1" t="n"/>
-      <c r="K21" s="1" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>376</v>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>static size_t copy_page_to_iter_pipe(struct page *page, size_t offset, size_t bytes,
 			 struct iov_iter *i)
@@ -4143,22 +3926,22 @@
 }</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>['CWE-284']</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>A flaw was found in the way the "flags" member of the new pipe buffer structure was lacking proper initialization in copy_page_to_iter_pipe and push_pipe functions in the Linux kernel and could thus contain stale values. An unprivileged local user could use this flaw to write to pages in the page cache backed by read only files and as such escalate their privileges on the system.</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>### Analysis of the Provided Code
 The function `copy_page_to_iter_pipe` is a static kernel function that handles copying data from a memory page into a pipe buffer, using an iterator (`iov_iter`) to track the current position in the pipe. The code is part of the Linux kernel's internal pipe handling logic and is designed to manage the allocation and merging of pipe buffers.
@@ -4191,125 +3974,22 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
-      <c r="G22" s="1" t="n"/>
-      <c r="H22" s="1" t="n"/>
-      <c r="I22" s="1" t="n"/>
-      <c r="J22" s="1" t="n"/>
-      <c r="K22" s="1" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>404</v>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    QueueHandle_t xQueueGenericCreate( const UBaseType_t uxQueueLength,
-                                       const UBaseType_t uxItemSize,
-                                       const uint8_t ucQueueType )
-    {
-        Queue_t * pxNewQueue;
-        size_t xQueueSizeInBytes;
-        uint8_t * pucQueueStorage;
-        configASSERT( uxQueueLength &gt; ( UBaseType_t ) 0 );
-        /* Allocate enough space to hold the maximum number of items that
-         * can be in the queue at any time.  It is valid for uxItemSize to be
-         * zero in the case the queue is used as a semaphore. */
-        xQueueSizeInBytes = ( size_t ) ( uxQueueLength * uxItemSize ); /*lint !e961 MISRA exception as the casts are only redundant for some ports. */
-        /* Check for multiplication overflow. */
-        configASSERT( ( uxItemSize == 0 ) || ( uxQueueLength == ( xQueueSizeInBytes / uxItemSize ) ) );
-        /* Check for addition overflow. */
-        configASSERT( ( sizeof( Queue_t ) + xQueueSizeInBytes ) &gt;  xQueueSizeInBytes );
-        /* Allocate the queue and storage area.  Justification for MISRA
-         * deviation as follows:  pvPortMalloc() always ensures returned memory
-         * blocks are aligned per the requirements of the MCU stack.  In this case
-         * pvPortMalloc() must return a pointer that is guaranteed to meet the
-         * alignment requirements of the Queue_t structure - which in this case
-         * is an int8_t *.  Therefore, whenever the stack alignment requirements
-         * are greater than or equal to the pointer to char requirements the cast
-         * is safe.  In other cases alignment requirements are not strict (one or
-         * two bytes). */
-        pxNewQueue = ( Queue_t * ) pvPortMalloc( sizeof( Queue_t ) + xQueueSizeInBytes ); /*lint !e9087 !e9079 see comment above. */
-        if( pxNewQueue != NULL )
-        {
-            /* Jump past the queue structure to find the location of the queue
-             * storage area. */
-            pucQueueStorage = ( uint8_t * ) pxNewQueue;
-            pucQueueStorage += sizeof( Queue_t ); /*lint !e9016 Pointer arithmetic allowed on char types, especially when it assists conveying intent. */
-            #if ( configSUPPORT_STATIC_ALLOCATION == 1 )
-                {
-                    /* Queues can be created either statically or dynamically, so
-                     * note this task was created dynamically in case it is later
-                     * deleted. */
-                    pxNewQueue-&gt;ucStaticallyAllocated = pdFALSE;
-                }
-            #endif /* configSUPPORT_STATIC_ALLOCATION */
-            prvInitialiseNewQueue( uxQueueLength, uxItemSize, pucQueueStorage, ucQueueType, pxNewQueue );
-        }
-        else
-        {
-            traceQUEUE_CREATE_FAILED( ucQueueType );
-            mtCOVERAGE_TEST_MARKER();
-        }
-        return pxNewQueue;
-    }-</t>
-        </is>
-      </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="n"/>
-      <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="inlineStr">
-        <is>
-          <t>### Analysis of the Provided Code
-The function `xQueueGenericCreate` is part of the FreeRTOS kernel and is responsible for dynamically creating a queue. It takes three parameters: `uxQueueLength` (the maximum number of items in the queue), `uxItemSize` (the size of each item in bytes), and `ucQueueType` (the type of queue, e.g., blocking, FIFO, etc.). The function performs several critical checks and allocations to ensure safe and correct behavior.
----
-### Key Security Considerations
-1. **Input Validation and Overflow Checks**:
-   - **Multiplication Overflow Check**:
-     The code calculates `xQueueSizeInBytes = uxQueueLength * uxItemSize` and checks for overflow using:
-     ```c
-     configASSERT( ( uxItemSize == 0 ) || ( uxQueueLength == ( xQueueSizeInBytes / uxItemSize ) ) );
-     ```
-     This ensures that the multiplication does not overflow. If `uxItemSize` is zero (valid for semaphores), the check is skipped. Otherwise, it verifies that the division of the resulting size by `uxItemSize` returns the original `uxQueueLength`, which would not be the case if an overflow occurred. This is a robust and correct way to detect multiplication overflow.
-   - **Addition Overflow Check**:
-     The code checks for overflow in the total memory allocation size:
-     ```c
-     configASSERT( ( sizeof( Queue_t ) + xQueueSizeInBytes ) &gt; xQueueSizeInBytes );
-     ```
-     This ensures that the sum of `sizeof(Queue_t)` and `xQueueSizeInBytes` does not overflow. Since `sizeof(Queue_t)` is always positive, the sum will be greater than `xQueueSizeInBytes` unless an overflow occurs. This is a standard and effective way to detect addition overflow in unsigned arithmetic.
-2. **Memory Allocation**:
-   - The function uses `pvPortMalloc` to allocate memory for the queue structure and its storage area. The allocation size is `sizeof(Queue_t) + xQueueSizeInBytes`, which is correct and aligns with the structure layout.
-   - The code checks if the allocation fails (`pxNewQueue == NULL`) and logs an error in that case, which is a good practice.
-3. **Pointer Arithmetic and Alignment**:
-   - The code uses pointer arithmetic to locate the queue storage area after the `Queue_t` structure. This is valid in C, especially when using `uint8_t*` (which is effectively a byte pointer), and the comment justifies the MISRA deviation for alignment, which is acceptable in this context.
-4. **Static vs. Dynamic Allocation**:
-   - The code includes a conditional block for static allocation support (`configSUPPORT_STATIC_ALLOCATION`), which is handled correctly by setting `ucStaticallyAllocated` to `pdFALSE` for dynamically created queues.
-5. **Initialization**:
-   - The function calls `prvInitialiseNewQueue` to initialize the queue structure and storage. While the implementation of this function is not visible, the call is made only if the allocation is successful, which is correct.
----
-### Conclusion
-The code includes comprehensive checks for **multiplication and addition overflows**, proper **memory allocation**, and **safe pointer arithmetic**. It also handles **edge cases** such as `uxItemSize == 0` (used for semaphores) and **allocation failure** gracefully. The use of `configASSERT` ensures that invalid inputs or overflow conditions are caught during development, and the code is structured to prevent memory-related vulnerabilities such as buffer overflows or incorrect memory allocation.
-While the effectiveness of `configASSERT` depends on whether assertions are enabled in the build configuration, the code as written includes these checks and is designed to be secure under normal development and testing conditions.
----
-### Final Answer
-**(2) NO: No vulnerability.**</t>
-        </is>
-      </c>
-      <c r="G23" s="1" t="n"/>
-      <c r="H23" s="1" t="n"/>
-      <c r="I23" s="1" t="n"/>
-      <c r="J23" s="1" t="n"/>
-      <c r="K23" s="1" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
+    <row r="20">
+      <c r="A20" s="2" t="n">
         <v>420</v>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>fiber_switch(mrb_state *mrb, mrb_value self, mrb_int len, const mrb_value *a, mrb_bool resume, mrb_bool vmexec)
 {
@@ -4373,22 +4053,22 @@
 }</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>vulnerable</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>['CWE-703']</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>NULL Pointer Dereference in GitHub repository mruby/mruby prior to 3.2.</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if there's a vulnerability.
 **Code Overview**
@@ -4422,17 +4102,22 @@
 * If there are specific vulnerability types (e.g., timing attacks, side-channel vulnerabilities) not immediately apparent from the code, a more detailed analysis with those in mind might be necessary.</t>
         </is>
       </c>
-      <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="1" t="n"/>
-      <c r="J24" s="1" t="n"/>
-      <c r="K24" s="1" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
+    <row r="21">
+      <c r="A21" s="2" t="n">
         <v>426</v>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>change_indent(
     int		type,
@@ -4622,14 +4307,14 @@
 }</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D25" s="1" t="n"/>
-      <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -4645,17 +4330,22 @@
 **Conclusion:** The code contains a vulnerability due to improper validation of the allocation size, which can lead to memory corruption. This is a critical issue that requires fixing by adding checks to ensure `i` is non-negative before allocation.</t>
         </is>
       </c>
-      <c r="G25" s="1" t="n"/>
-      <c r="H25" s="1" t="n"/>
-      <c r="I25" s="1" t="n"/>
-      <c r="J25" s="1" t="n"/>
-      <c r="K25" s="1" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
+    <row r="22">
+      <c r="A22" s="2" t="n">
         <v>437</v>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>suggest_trie_walk(
     suginfo_T	*su,
@@ -5736,14 +5426,14 @@
 		mch_memmove(p + fl + tl, p</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D26" s="1" t="n"/>
-      <c r="E26" s="1" t="n"/>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>The provided code contains a potential **stack buffer overflow vulnerability** due to insufficient bounds checking on the `depth` variable when accessing the `stack` array.
 ### Key Analysis:
@@ -5772,17 +5462,22 @@
 **Answer:** YES</t>
         </is>
       </c>
-      <c r="G26" s="1" t="n"/>
-      <c r="H26" s="1" t="n"/>
-      <c r="I26" s="1" t="n"/>
-      <c r="J26" s="1" t="n"/>
-      <c r="K26" s="1" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>vulnerable</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
+    <row r="23">
+      <c r="A23" s="2" t="n">
         <v>459</v>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>static bool tipc_crypto_key_rcv(struct tipc_crypto *rx, struct tipc_msg *hdr)
 {
@@ -5836,14 +5531,14 @@
 }</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>safe</t>
         </is>
       </c>
-      <c r="D27" s="1" t="n"/>
-      <c r="E27" s="1" t="n"/>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
@@ -5876,11 +5571,16 @@
 **Note**: This analysis is based solely on the provided code snippet. The overall security of the system also depends on the correctness and security of the surrounding code, which is not analyzed here.</t>
         </is>
       </c>
-      <c r="G27" s="1" t="n"/>
-      <c r="H27" s="1" t="n"/>
-      <c r="I27" s="1" t="n"/>
-      <c r="J27" s="1" t="n"/>
-      <c r="K27" s="1" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>